<commit_message>
Re-cut target companies around conviction and skill ramp
Reorganizes the target company tab into six lanes ordered by field
conviction rather than company prestige, and adds a "what skill it ramps"
column so each row states what the job would teach.

Adds 14 companies, notably AI-recruiting (Juicebox, Jobright, Micro1,
Paraform, Surge), workforce AI adoption (Section, Maven, Reforge), an LA
AI consultancy (AE Studio), and a lane for stated personal interests
(Chess.com, WHOOP, Oura, HeyGen, Splice, Snap, GumGum).

Demotes six that were included for proximity or prestige rather than fit
(Scopely, FloQast, Anduril, Block, Lightcast, and a second-tier group),
keeping them visible with the reason stated.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RRApM4jepKAL4DBnTT6Rsj
</commit_message>
<xml_diff>
--- a/career/Miles_Tipton_MASTER_Tracker_Aug1_2026_VERIFIED.xlsx
+++ b/career/Miles_Tipton_MASTER_Tracker_Aug1_2026_VERIFIED.xlsx
@@ -17,7 +17,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'✅ Job Tracker (Verified)'!$A$2:$K$36</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'🏢 Target Companies'!$A$2:$H$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'🏢 Target Companies'!$A$2:$I$64</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2657,23 +2657,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H54"/>
+  <dimension ref="A1:I68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="74" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="66" customWidth="1" min="6" max="6"/>
     <col width="34" customWidth="1" min="7" max="7"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="38" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>TARGET COMPANIES — companies worth wanting, grouped by the five lanes your work actually sits in</t>
+          <t>TARGET COMPANIES v2 — re-cut around conviction and skill ramp, not company prestige</t>
         </is>
       </c>
     </row>
@@ -2705,44 +2706,49 @@
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>Why this one should excite you</t>
+          <t>Why this one should excite YOU specifically</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
+          <t>What skill it ramps</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
           <t>Roles to watch</t>
         </is>
       </c>
-      <c r="H2" s="5" t="inlineStr">
+      <c r="I2" s="5" t="inlineStr">
         <is>
           <t>Careers page</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="22" customHeight="1">
+    <row r="3" ht="26" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>LANE 1 — CAREER &amp; LABOR-MARKET INTELLIGENCE  ·  this is UPath's category. Working here is paid market research.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="60" customHeight="1">
+          <t>LANE 1 — AI × HIRING AND LABOR MARKETS  ·  THE FIELD TO DOUBLE DOWN IN. This stopped being a theme and became a funded category: ten US AI-recruiting startups raised $656M between July 2025 and July 2026. You are already building in it. Get paid to be inside it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="48" customHeight="1">
       <c r="A4" s="6" t="n">
         <v>1</v>
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>ZipRecruiter</t>
+          <t>Mercor</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>Santa Monica, CA</t>
+          <t>San Francisco</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>LA — hybrid</t>
+          <t>Remote-limited</t>
         </is>
       </c>
       <c r="E4" s="8" t="inlineStr">
@@ -2752,17 +2758,22 @@
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>The obvious one, and it was missing entirely from the original tracker. A labor-market company headquartered 20 minutes from you, with roughly 20 openings near Santa Monica including sales-enablement roles that want Salesforce, Sales Cloud, and dashboarding. Everything you would learn about how job matching actually works at scale is directly reusable for UPath.</t>
+          <t>The category leader. $10B valuation Oct 2025, in talks at $20B nine months later, ~200 employees, ~65 open roles, 30,000+ contractors paid $1.5M+ a day. They turned 'match experts to work' into a real market. That is UPath's mechanism, at scale, with a balance sheet.</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
         <is>
-          <t>Sales Enablement · Account Executive · RevOps</t>
-        </is>
-      </c>
-      <c r="H4" s="9" t="inlineStr">
-        <is>
-          <t>https://www.ziprecruiter.com/careers</t>
+          <t>Marketplace dynamics · supply/demand matching · AI-era labor economics</t>
+        </is>
+      </c>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>GTM · Ops · Expert Network</t>
+        </is>
+      </c>
+      <c r="I4" s="9" t="inlineStr">
+        <is>
+          <t>https://www.mercor.com/careers/</t>
         </is>
       </c>
     </row>
@@ -2772,7 +2783,7 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>Mercor</t>
+          <t>Juicebox (PeopleGPT)</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
@@ -2782,7 +2793,7 @@
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>Remote-limited</t>
+          <t>Remote-friendly</t>
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr">
@@ -2792,32 +2803,37 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>The most interesting company in your entire category right now. $10B valuation as of Oct 2025, in talks at $20B, ~200 employees, ~65 open roles, and 30,000+ contractors being paid over $1.5M a day. They matched experts to AI labs — which is a labor market with an AI-era matching layer. That is your thesis, funded.</t>
+          <t>The hottest thing in this lane and it was nowhere in v1. $80M Series B in March 2026 at an $850M valuation, DST / Sequoia / Coatue / YC, ARR tripled since July 2025, ~5,000 customers, 800M candidate profiles searchable in plain English. Natural-language search over a labor-market graph is the exact problem shape you are working on.</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
-          <t>GTM · Ops · Expert Network</t>
-        </is>
-      </c>
-      <c r="H5" s="9" t="inlineStr">
-        <is>
-          <t>https://www.mercor.com/careers/</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="48" customHeight="1">
+          <t>Semantic search over people data · AI-native GTM · PLG in HR tech</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>GTM Engineer · AE · Solutions</t>
+        </is>
+      </c>
+      <c r="I5" s="9" t="inlineStr">
+        <is>
+          <t>https://juicebox.ai/careers</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="72" customHeight="1">
       <c r="A6" s="6" t="n">
         <v>3</v>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Revelio Labs</t>
+          <t>Jobright.ai</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>Santa Clara, CA</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
@@ -2827,22 +2843,27 @@
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>VERIFIED ACTIVE</t>
+          <t>VERIFIED HIRING</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>Workforce intelligence built from 5B+ job postings across 30M companies. On July 28, 2026 they launched an AI Labor Market Tracker measuring AI's real impact on employment. That is literally the data layer UPath needs. Even a customer-facing role here would teach you how this data gets sold and to whom.</t>
+          <t>The closest thing to a direct UPath peer on this list — and that is a feature, not a conflict. 88 people, 520,000+ users, growing 30x year over year, $7.7M raised with Indeed's venture arm participating. An AI career agent that finds, tailors and submits applications. Working here would teach you exactly which parts of that thesis hold up commercially and which do not.</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
-          <t>Solutions Consultant · CS · Sales</t>
-        </is>
-      </c>
-      <c r="H6" s="9" t="inlineStr">
-        <is>
-          <t>https://www.reveliolabs.com/careers</t>
+          <t>Career-agent product mechanics · what users actually pay for</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>GTM · Growth · Partnerships</t>
+        </is>
+      </c>
+      <c r="I6" s="9" t="inlineStr">
+        <is>
+          <t>https://jobright.ai/</t>
         </is>
       </c>
     </row>
@@ -2852,37 +2873,42 @@
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Lightcast</t>
+          <t>Micro1</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>Remote-first</t>
+          <t>Palo Alto, CA</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>Remote</t>
+          <t>Remote-friendly</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>ACTIVE</t>
+          <t>VERIFIED HIRING</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>The incumbent in labor-market intelligence — 18 billion data points across 165 countries. Less exciting than Revelio, but far bigger, and they sell to governments, universities, and enterprises. Good place to learn how workforce data is actually packaged and priced.</t>
+          <t>Quietly one of the fastest growers anywhere: $300M annualized revenue in April 2026, up from $125M at the end of 2025. Three products — a talent marketplace, an AI recruiter called Zara, and expert data work. Human intelligence as infrastructure for AI systems.</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
-          <t>Solutions Consultant · Client Success</t>
-        </is>
-      </c>
-      <c r="H7" s="9" t="inlineStr">
-        <is>
-          <t>https://lightcast.io/about/careers</t>
+          <t>AI-assisted vetting · expert-network operations · revenue at speed</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>GTM · Expert Ops · Solutions</t>
+        </is>
+      </c>
+      <c r="I7" s="9" t="inlineStr">
+        <is>
+          <t>https://www.micro1.ai/careers</t>
         </is>
       </c>
     </row>
@@ -2892,7 +2918,7 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Handshake</t>
+          <t>Paraform</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
@@ -2907,117 +2933,132 @@
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>VERIFIED HIRING</t>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>20M knowledge workers, 1,600 institutions, and a stated mission of a path to a career regardless of where you went to school — which is close to how you describe UPath. Their newer Handshake AI arm does expert data work too, so there are two doors in.</t>
+          <t>Agentic hiring — specialist recruiters and AI working the same req, average 12 days to hire, filling roles for Palantir, Rippling and Cognition across 1,000+ companies. Small enough that a generalist who can sell, research and build workflows is obviously useful.</t>
         </is>
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>GTM · Partnerships · Handshake AI</t>
-        </is>
-      </c>
-      <c r="H8" s="9" t="inlineStr">
-        <is>
-          <t>https://joinhandshake.com/careers/</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="48" customHeight="1">
+          <t>Human-in-the-loop AI workflows · recruiter economics</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>GTM · Recruiter Ops</t>
+        </is>
+      </c>
+      <c r="I8" s="9" t="inlineStr">
+        <is>
+          <t>https://www.paraform.com/careers</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="46" customHeight="1">
       <c r="A9" s="6" t="n">
         <v>6</v>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Correlation One</t>
+          <t>Surge AI</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>Remote</t>
+          <t>San Francisco</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>Remote</t>
+          <t>Remote-friendly</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">
         <is>
-          <t>VERIFIED HIRING</t>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>Already in your tracker twice over. Worth naming here as a company, not just a job: they have trained 500,000+ people across 11 countries in AI and data. Two contract doors are open right now (AI Coach and Career Success Coach) and both put you in front of career-changers all day.</t>
+          <t>Took the frontier-lab data crown after Meta absorbed 49% of Scale in June 2025. Notoriously lean, notoriously profitable. The commercial side of frontier-model data work.</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
-          <t>AI Coach · Career Success Coach</t>
-        </is>
-      </c>
-      <c r="H9" s="9" t="inlineStr">
-        <is>
-          <t>https://job-boards.greenhouse.io/correlationone</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="46" customHeight="1">
+          <t>Frontier-lab buying behavior · expert data supply chains</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>GTM · Ops</t>
+        </is>
+      </c>
+      <c r="I9" s="9" t="inlineStr">
+        <is>
+          <t>https://www.surgehq.ai/careers</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="60" customHeight="1">
       <c r="A10" s="6" t="n">
         <v>7</v>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Teal HQ</t>
+          <t>ZipRecruiter</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Remote</t>
+          <t>Santa Monica, CA</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>Remote</t>
+          <t>LA — hybrid</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>ACTIVE</t>
+          <t>VERIFIED HIRING</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>Career-management software for job seekers — the consumer-tools end of what UPath does. Small, so the opening rate is low, but the overlap is near-total and that makes for a genuinely strong cover letter.</t>
+          <t>The incumbent in your own city. ~20 openings near Santa Monica including sales-enablement roles wanting Salesforce, Sales Cloud and dashboarding. Less exciting than Mercor or Juicebox — but it is the only labor-market company you can drive to, and matching at their scale is a genuine education.</t>
         </is>
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>GTM · Growth · Partnerships</t>
-        </is>
-      </c>
-      <c r="H10" s="9" t="inlineStr">
-        <is>
-          <t>https://www.tealhq.com/about</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="46" customHeight="1">
+          <t>Marketplace liquidity · enablement systems at scale</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>Sales Enablement · AE · RevOps</t>
+        </is>
+      </c>
+      <c r="I10" s="9" t="inlineStr">
+        <is>
+          <t>https://www.ziprecruiter.com/careers</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="48" customHeight="1">
       <c r="A11" s="6" t="n">
         <v>8</v>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Eightfold AI</t>
+          <t>Revelio Labs</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Santa Clara, CA</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
@@ -3027,69 +3068,79 @@
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>ACTIVE</t>
+          <t>VERIFIED ACTIVE</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>Talent-intelligence platform selling AI-driven matching to large enterprises. The enterprise mirror of UPath: same problem, opposite customer. A solutions role here would teach you the objection set.</t>
+          <t>Workforce intelligence from 5B+ postings across 30M companies, and on July 28, 2026 they shipped an AI Labor Market Tracker measuring AI's actual effect on employment. If you ever want to argue about AI disruption with data instead of takes, this is the building.</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>Solutions Consultant · Sales Engineer</t>
-        </is>
-      </c>
-      <c r="H11" s="9" t="inlineStr">
-        <is>
-          <t>https://eightfold.ai/careers/</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>LANE 2 — GTM ENGINEERING &amp; AI-NATIVE SALES TECH  ·  the highest-leverage lane you are not yet aiming at.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="84" customHeight="1">
-      <c r="A13" s="6" t="n">
+          <t>Labor-market data modeling · how workforce data is sold</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>Solutions Consultant · CS · Sales</t>
+        </is>
+      </c>
+      <c r="I11" s="9" t="inlineStr">
+        <is>
+          <t>https://www.reveliolabs.com/careers</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="46" customHeight="1">
+      <c r="A12" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="7" t="inlineStr">
-        <is>
-          <t>Clay</t>
-        </is>
-      </c>
-      <c r="C13" s="7" t="inlineStr">
-        <is>
-          <t>New York / Remote</t>
-        </is>
-      </c>
-      <c r="D13" s="7" t="inlineStr">
-        <is>
-          <t>Remote</t>
-        </is>
-      </c>
-      <c r="E13" s="8" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Handshake</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>San Francisco</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>Remote-friendly</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
         <is>
           <t>VERIFIED HIRING</t>
         </is>
       </c>
-      <c r="F13" s="7" t="inlineStr">
-        <is>
-          <t>Read this row twice. GTM Engineer is a real, fast-forming job title — postings went from ~1,400 in mid-2025 to 3,000+ by January 2026, up 205% year over year, at $132K–$241K. The job is: build the enrichment pipelines, automated plays, and no-code workflows that power outbound. Clay, Make, Zapier, APIs, ICP research, cold email. That is a description of what you already do at Social Hog with a salary attached, and it was not on your Top 20 at all. Clay also runs a dedicated GTM job board.</t>
-        </is>
-      </c>
-      <c r="G13" s="7" t="inlineStr">
-        <is>
-          <t>GTM Engineer · GTM Solutions Engineer</t>
-        </is>
-      </c>
-      <c r="H13" s="9" t="inlineStr">
-        <is>
-          <t>https://www.clay.com/careers</t>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>20M knowledge workers, 1,600 institutions, and a mission statement close enough to yours to be awkward. Two doors: the core marketplace, and Handshake AI doing expert data work.</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>Early-career market mechanics · two-sided marketplace GTM</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>GTM · Partnerships · Handshake AI</t>
+        </is>
+      </c>
+      <c r="I12" s="9" t="inlineStr">
+        <is>
+          <t>https://joinhandshake.com/careers/</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>LANE 2 — AI ENABLEMENT &amp; WORKFORCE TRANSFORMATION  ·  the job is literally 'help humans adapt to AI'. Your thesis, as a salaried function.</t>
         </is>
       </c>
     </row>
@@ -3099,57 +3150,62 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>Nooks</t>
+          <t>Section</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>SF / Seattle</t>
+          <t>New York / Remote</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>Hybrid</t>
+          <t>Remote-friendly</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
         <is>
-          <t>VERIFIED HIRING</t>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>AI outbound platform — 1,500+ customers including Notion, HubSpot and Rippling, $70M+ raised from Kleiner Perkins, hiring across engineering, product and GTM, and standing up a new Seattle engineering office. You have personally cold-called with tools like this; that is a real differentiator in their interview.</t>
+          <t>Read the one-line description twice: they help enterprises MEASURE AND ACCELERATE AI ADOPTION ACROSS THEIR WORKFORCE. That is AI disruption, career change and enablement in a single product. Of everything I found in this pass, this is the tightest thesis match to how you describe your own work.</t>
         </is>
       </c>
       <c r="G14" s="7" t="inlineStr">
         <is>
-          <t>GTM · SDR · Solutions</t>
-        </is>
-      </c>
-      <c r="H14" s="9" t="inlineStr">
-        <is>
-          <t>https://www.nooks.ai/careers</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="46" customHeight="1">
+          <t>AI adoption measurement · workforce change management</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>Enablement · Solutions · GTM</t>
+        </is>
+      </c>
+      <c r="I14" s="9" t="inlineStr">
+        <is>
+          <t>https://www.sections.school/</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="48" customHeight="1">
       <c r="A15" s="6" t="n">
         <v>11</v>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Kixie</t>
+          <t>Maven</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>Santa Monica, CA</t>
+          <t>Remote</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>LA — on-site</t>
+          <t>Remote</t>
         </is>
       </c>
       <c r="E15" s="8" t="inlineStr">
@@ -3159,37 +3215,42 @@
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>Also in your tracker as an SDR row. As a company it belongs here: sales-engagement tooling for HubSpot, Salesforce and Pipedrive, based in Santa Monica. Selling the dialer you already live in.</t>
+          <t>Cohort-based courses taught by practitioners, 5 open roles on their Greenhouse board, explicitly 'building the university of tomorrow'. The AI-upskilling category runs through them. Adjacent to content, teaching and career change — three things you already do for free.</t>
         </is>
       </c>
       <c r="G15" s="7" t="inlineStr">
         <is>
-          <t>SDR · Solutions</t>
-        </is>
-      </c>
-      <c r="H15" s="9" t="inlineStr">
-        <is>
-          <t>https://jobs.lever.co/kixie</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="46" customHeight="1">
+          <t>Cohort economics · creator/expert GTM · course marketplaces</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>GTM · Partnerships · Instructor Ops</t>
+        </is>
+      </c>
+      <c r="I15" s="9" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/maven</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="48" customHeight="1">
       <c r="A16" s="6" t="n">
         <v>12</v>
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>Gong</t>
+          <t>Reforge</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>SF / Remote</t>
+          <t>Remote</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>Remote-friendly</t>
+          <t>Remote</t>
         </is>
       </c>
       <c r="E16" s="8" t="inlineStr">
@@ -3199,17 +3260,22 @@
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
-          <t>Revenue intelligence — AI that reads sales conversations. Big, well-run, and the product is the clearest commercial expression of 'AI applied to sales conversations', which is your stated intersection.</t>
+          <t>Career development for senior tech operators — 78% PM placement within six months versus 54% for Product School. The premium end of career acceleration, and a masterclass in how expertise gets packaged and sold.</t>
         </is>
       </c>
       <c r="G16" s="7" t="inlineStr">
         <is>
-          <t>Solutions Consultant · Sales Engineer</t>
-        </is>
-      </c>
-      <c r="H16" s="9" t="inlineStr">
-        <is>
-          <t>https://www.gong.io/careers/</t>
+          <t>Positioning · premium pricing · career-outcome products</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>GTM · Partnerships · Programs</t>
+        </is>
+      </c>
+      <c r="I16" s="9" t="inlineStr">
+        <is>
+          <t>https://www.reforge.com/careers</t>
         </is>
       </c>
     </row>
@@ -3219,12 +3285,12 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Apollo.io</t>
+          <t>Correlation One</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>Remote-first</t>
+          <t>Remote</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
@@ -3234,22 +3300,27 @@
       </c>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>ACTIVE</t>
+          <t>VERIFIED HIRING</t>
         </is>
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>You already use Apollo — it is listed in your own sales-tools profile. Being a genuine power user of the product you would be selling shortens the ramp story more than any bullet point can.</t>
+          <t>500,000+ people trained across 11 countries. Two contract doors open now — AI Coach and Career Success Coach — and both put you in a room with career-changers every week. You already have the interview.</t>
         </is>
       </c>
       <c r="G17" s="7" t="inlineStr">
         <is>
-          <t>SDR · AE SMB · Solutions</t>
-        </is>
-      </c>
-      <c r="H17" s="9" t="inlineStr">
-        <is>
-          <t>https://www.apollo.io/careers</t>
+          <t>Cohort coaching · career-change patterns at volume</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>AI Coach · Career Success Coach</t>
+        </is>
+      </c>
+      <c r="I17" s="9" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/correlationone</t>
         </is>
       </c>
     </row>
@@ -3259,12 +3330,12 @@
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>Common Room</t>
+          <t>Kyndryl</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>Seattle / Remote</t>
+          <t>Remote</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
@@ -3274,129 +3345,144 @@
       </c>
       <c r="E18" s="8" t="inlineStr">
         <is>
-          <t>ACTIVE</t>
+          <t>VERIFIED HIRING</t>
         </is>
       </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
-          <t>Signal-based GTM — pulling buying intent out of scattered data. Adjacent to Clay, smaller, and hungry for people who can think in workflows rather than scripts.</t>
+          <t>Not exciting. Is verified, salaried, remote and real — live Workday req R-61971 for AI Enablement Specialist. Enterprise AI adoption and training. Treat it as the floor under the more interesting bets.</t>
         </is>
       </c>
       <c r="G18" s="7" t="inlineStr">
         <is>
-          <t>GTM Engineer · Solutions</t>
-        </is>
-      </c>
-      <c r="H18" s="9" t="inlineStr">
-        <is>
-          <t>https://www.commonroom.io/careers/</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>LANE 3 — SMB, LOCAL SEARCH &amp; MAIN STREET  ·  Social Hog and Built for Main Street are your unfair advantage here.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="60" customHeight="1">
+          <t>Enterprise change management · structured enablement</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>AI Enablement Specialist</t>
+        </is>
+      </c>
+      <c r="I18" s="9" t="inlineStr">
+        <is>
+          <t>https://kyndryl.wd5.myworkdayjobs.com/KyndrylProfessionalCareers</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="72" customHeight="1">
+      <c r="A19" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>AE Studio</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>Venice, CA</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>LA — hybrid</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>VERIFIED HIRING</t>
+        </is>
+      </c>
+      <c r="F19" s="7" t="inlineStr">
+        <is>
+          <t>The best-kept secret in LA tech and a genuine omission from v1. Venice office, fully bootstrapped — no VC, no PE, they sell work at a profit and pay people from it. Builds production AI for Samsung, Walmart and Berkshire Hathaway while also doing frontier alignment research, and they explicitly hire 'researchers, engineers and operators who ship hard things'. The word OPERATORS is the opening.</t>
+        </is>
+      </c>
+      <c r="G19" s="7" t="inlineStr">
+        <is>
+          <t>Real AI implementation across many clients — fastest skill ramp in LA</t>
+        </is>
+      </c>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>Operator · Product Lead · BD</t>
+        </is>
+      </c>
+      <c r="I19" s="9" t="inlineStr">
+        <is>
+          <t>https://ae.studio/join-us</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="48" customHeight="1">
       <c r="A20" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>SOCi</t>
+          <t>Glean</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>San Diego, CA</t>
+          <t>Remote (US)</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>SoCal / hybrid</t>
+          <t>Remote</t>
         </is>
       </c>
       <c r="E20" s="8" t="inlineStr">
         <is>
-          <t>VERIFIED ACTIVE</t>
+          <t>VERIFIED HIRING</t>
         </is>
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
-          <t>The single most on-thesis company in this file. 632 employees, and their whole product is an agentic AI workforce that manages local search, listings, reviews and social for 1,000+ multi-location brands — Social Hog, at enterprise scale, automated. You can speak to the pain in their pitch deck from memory because you have heard it on the phone from actual owners.</t>
+          <t>Enterprise AI search and agents, remote US Solutions Engineers at $110K–$235K. The SE job is demos, architecture explanation and proof-of-value — your Inbenta work one technology generation later. Current reqs skew senior; watch for a mid-market opening.</t>
         </is>
       </c>
       <c r="G20" s="7" t="inlineStr">
         <is>
-          <t>Solutions Consultant · SDR · CS</t>
-        </is>
-      </c>
-      <c r="H20" s="9" t="inlineStr">
-        <is>
-          <t>https://www.soci.ai/careers/</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="60" customHeight="1">
-      <c r="A21" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="B21" s="7" t="inlineStr">
-        <is>
-          <t>Tebra (Kareo + PatientPop)</t>
-        </is>
-      </c>
-      <c r="C21" s="7" t="inlineStr">
-        <is>
-          <t>Newport Beach, CA</t>
-        </is>
-      </c>
-      <c r="D21" s="7" t="inlineStr">
-        <is>
-          <t>SoCal / hybrid</t>
-        </is>
-      </c>
-      <c r="E21" s="8" t="inlineStr">
-        <is>
-          <t>VERIFIED HIRING</t>
-        </is>
-      </c>
-      <c r="F21" s="7" t="inlineStr">
-        <is>
-          <t>Newport Beach, roughly an hour from you, active Greenhouse board. Their PatientPop side sells digital presence, online reputation and local visibility to independent medical practices with under 10 providers. That is Built for Main Street pointed at doctors. Your Google Business Profile diagnostics translate directly into their discovery call.</t>
-        </is>
-      </c>
-      <c r="G21" s="7" t="inlineStr">
-        <is>
-          <t>Solutions Consultant · SDR · CS</t>
-        </is>
-      </c>
-      <c r="H21" s="9" t="inlineStr">
-        <is>
-          <t>https://job-boards.greenhouse.io/tebra</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="46" customHeight="1">
+          <t>Enterprise AI deployment · POV/POC motion</t>
+        </is>
+      </c>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>Solutions Engineer</t>
+        </is>
+      </c>
+      <c r="I20" s="9" t="inlineStr">
+        <is>
+          <t>https://www.glean.com/careers</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>LANE 3 — GTM ENGINEERING  ·  the skill to ramp in the next 90 days. Highest pay-to-difficulty ratio available to you right now.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="72" customHeight="1">
       <c r="A22" s="6" t="n">
         <v>17</v>
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>Housecall Pro</t>
+          <t>Clay</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>San Diego, CA</t>
+          <t>New York / Remote</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>Remote-first</t>
+          <t>Remote</t>
         </is>
       </c>
       <c r="E22" s="8" t="inlineStr">
@@ -3406,37 +3492,42 @@
       </c>
       <c r="F22" s="7" t="inlineStr">
         <is>
-          <t>Remote-first with San Diego and Denver offices, currently posting a remote US Inside Sales Rep. Sells to plumbers, electricians and HVAC contractors — the exact owner profile you cold call.</t>
+          <t>The keystone. GTM Engineer went from ~1,400 postings mid-2025 to 3,000+ by January 2026, up 205% year over year, posted at $132K–$241K. The job is enrichment pipelines, automated plays, APIs and outbound systems — described in the field as 'half commercial thinker, half builder'. That is your Social Hog workflow with a salary. Clay also runs the category's dedicated job board.</t>
         </is>
       </c>
       <c r="G22" s="7" t="inlineStr">
         <is>
-          <t>Inside Sales · CS · Sales Training</t>
-        </is>
-      </c>
-      <c r="H22" s="9" t="inlineStr">
-        <is>
-          <t>https://www.housecallpro.com/careers/</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="46" customHeight="1">
+          <t>THE core skill: Clay, Make, Zapier, n8n, APIs, enrichment, deliverability</t>
+        </is>
+      </c>
+      <c r="H22" s="7" t="inlineStr">
+        <is>
+          <t>GTM Engineer · GTM Solutions Engineer</t>
+        </is>
+      </c>
+      <c r="I22" s="9" t="inlineStr">
+        <is>
+          <t>https://www.clay.com/careers</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="48" customHeight="1">
       <c r="A23" s="6" t="n">
         <v>18</v>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>ServiceTitan</t>
+          <t>Nooks</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>Glendale, CA</t>
+          <t>SF / Seattle</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>LA — hybrid</t>
+          <t>Hybrid</t>
         </is>
       </c>
       <c r="E23" s="8" t="inlineStr">
@@ -3446,17 +3537,22 @@
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
-          <t>The biggest home-services software company in the country, headquartered in Glendale. Also the most credible LA-based launchpad on this list: ex-ServiceTitan people show up on the founding teams of companies like Owner.com.</t>
+          <t>AI outbound platform, 1,500+ customers including Notion, HubSpot and Rippling, $70M+ from Kleiner Perkins, hiring across engineering, product and GTM. You have personally cold-called with tools like this — that is a real edge in their interview loop, not a talking point.</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">
         <is>
-          <t>SDR · Solutions Consultant · CS</t>
-        </is>
-      </c>
-      <c r="H23" s="9" t="inlineStr">
-        <is>
-          <t>https://www.servicetitan.com/careers</t>
+          <t>AI-assisted outbound · dialer and sequencing systems</t>
+        </is>
+      </c>
+      <c r="H23" s="7" t="inlineStr">
+        <is>
+          <t>GTM · SDR · Solutions</t>
+        </is>
+      </c>
+      <c r="I23" s="9" t="inlineStr">
+        <is>
+          <t>https://www.nooks.ai/careers</t>
         </is>
       </c>
     </row>
@@ -3466,37 +3562,42 @@
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>Boulevard</t>
+          <t>Common Room</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>Los Angeles, CA</t>
+          <t>Seattle / Remote</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>LA — hybrid</t>
+          <t>Remote</t>
         </is>
       </c>
       <c r="E24" s="8" t="inlineStr">
         <is>
-          <t>VERIFIED HIRING</t>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="F24" s="7" t="inlineStr">
         <is>
-          <t>LA-headquartered, ~260 people, selling to salons, spas and self-care businesses. Local, venture-backed, and the buyer is one you have already talked to.</t>
+          <t>Signal-based GTM — pulling buying intent out of scattered community, product and social data. Adjacent to Clay, smaller, and receptive to people who think in workflows rather than scripts.</t>
         </is>
       </c>
       <c r="G24" s="7" t="inlineStr">
         <is>
-          <t>SDR · CS · Solutions</t>
-        </is>
-      </c>
-      <c r="H24" s="9" t="inlineStr">
-        <is>
-          <t>https://www.joinblvd.com/careers</t>
+          <t>Intent signals · data plumbing for revenue teams</t>
+        </is>
+      </c>
+      <c r="H24" s="7" t="inlineStr">
+        <is>
+          <t>GTM Engineer · Solutions</t>
+        </is>
+      </c>
+      <c r="I24" s="9" t="inlineStr">
+        <is>
+          <t>https://www.commonroom.io/careers/</t>
         </is>
       </c>
     </row>
@@ -3506,137 +3607,114 @@
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>Otter (CloudKitchens)</t>
+          <t>Apollo.io</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>Los Angeles, CA</t>
+          <t>Remote-first</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>LA — on-site</t>
+          <t>Remote</t>
         </is>
       </c>
       <c r="E25" s="8" t="inlineStr">
         <is>
-          <t>VERIFIED HIRING</t>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
-          <t>Restaurant operating software out of LA, with a Solutions Engineer role open right now. See the tracker — this is your best single application in the file.</t>
+          <t>Already in your own tool stack per your profile. Being a genuine power user of the product you would sell shortens the ramp story more than any bullet can.</t>
         </is>
       </c>
       <c r="G25" s="7" t="inlineStr">
         <is>
-          <t>Solutions Engineer · Implementation</t>
-        </is>
-      </c>
-      <c r="H25" s="9" t="inlineStr">
-        <is>
-          <t>https://job-boards.greenhouse.io/otter</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="46" customHeight="1">
-      <c r="A26" s="6" t="n">
+          <t>Data-driven prospecting at scale</t>
+        </is>
+      </c>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
+          <t>SDR · AE SMB · Solutions</t>
+        </is>
+      </c>
+      <c r="I25" s="9" t="inlineStr">
+        <is>
+          <t>https://www.apollo.io/careers</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>LANE 4 — FORWARD-DEPLOYED / APPLIED AI  ·  the 2–4 year target. Track these, build toward them, do not apply cold in August.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="72" customHeight="1">
+      <c r="A27" s="6" t="n">
         <v>21</v>
       </c>
-      <c r="B26" s="7" t="inlineStr">
-        <is>
-          <t>Owner.com</t>
-        </is>
-      </c>
-      <c r="C26" s="7" t="inlineStr">
-        <is>
-          <t>Remote-first (SF)</t>
-        </is>
-      </c>
-      <c r="D26" s="7" t="inlineStr">
-        <is>
-          <t>Remote</t>
-        </is>
-      </c>
-      <c r="E26" s="8" t="inlineStr">
-        <is>
-          <t>VERIFIED HIRING</t>
-        </is>
-      </c>
-      <c r="F26" s="7" t="inlineStr">
-        <is>
-          <t>Restaurant marketing and ordering for independent operators, 20,000+ owners served, ~$200M saved in fees. Explicitly hiring AEs with 1–2 years of SMB SaaS experience — the rare req written at your actual level.</t>
-        </is>
-      </c>
-      <c r="G26" s="7" t="inlineStr">
-        <is>
-          <t>AE · Outbound AE · CS Manager</t>
-        </is>
-      </c>
-      <c r="H26" s="9" t="inlineStr">
-        <is>
-          <t>https://jobs.ashbyhq.com/owner</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="46" customHeight="1">
-      <c r="A27" s="6" t="n">
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Palantir</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>Multiple US</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>ACTIVE — BENCHMARK</t>
+        </is>
+      </c>
+      <c r="F27" s="7" t="inlineStr">
+        <is>
+          <t>The company that invented the role. Their Forward Deployed Software Engineer, New Grad – Commercial req posts at $135K–$145K but is gated to Dec 2026 / Spring 2027 graduates, so that specific door is closed to a 2020 grad. Included because it is the benchmark: Python and SQL non-negotiable, data pipelining, production code, and running the customer meeting. That is the exact skill list to build toward.</t>
+        </is>
+      </c>
+      <c r="G27" s="7" t="inlineStr">
+        <is>
+          <t>The FDE standard: production code + customer ownership</t>
+        </is>
+      </c>
+      <c r="H27" s="7" t="inlineStr">
+        <is>
+          <t>FDSE (experienced tracks)</t>
+        </is>
+      </c>
+      <c r="I27" s="9" t="inlineStr">
+        <is>
+          <t>https://jobs.lever.co/palantir</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="48" customHeight="1">
+      <c r="A28" s="6" t="n">
         <v>22</v>
       </c>
-      <c r="B27" s="7" t="inlineStr">
-        <is>
-          <t>Yelp</t>
-        </is>
-      </c>
-      <c r="C27" s="7" t="inlineStr">
-        <is>
-          <t>Remote-first</t>
-        </is>
-      </c>
-      <c r="D27" s="7" t="inlineStr">
-        <is>
-          <t>Remote (West)</t>
-        </is>
-      </c>
-      <c r="E27" s="8" t="inlineStr">
-        <is>
-          <t>VERIFIED HIRING</t>
-        </is>
-      </c>
-      <c r="F27" s="7" t="inlineStr">
-        <is>
-          <t>90%+ of openings are remote. Local search is the whole company. If you ever want to argue about Google Business Profile ranking for a living, this is the building.</t>
-        </is>
-      </c>
-      <c r="G27" s="7" t="inlineStr">
-        <is>
-          <t>Inside Sales · Local Account Exec</t>
-        </is>
-      </c>
-      <c r="H27" s="9" t="inlineStr">
-        <is>
-          <t>https://www.yelp.careers/us/en</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="46" customHeight="1">
-      <c r="A28" s="6" t="n">
-        <v>23</v>
-      </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>Birdeye</t>
+          <t>Sierra AI</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>Palo Alto, CA</t>
+          <t>San Francisco</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>Remote-friendly</t>
+          <t>Hybrid</t>
         </is>
       </c>
       <c r="E28" s="8" t="inlineStr">
@@ -3646,471 +3724,569 @@
       </c>
       <c r="F28" s="7" t="inlineStr">
         <is>
-          <t>Reviews, listings and messaging AI for multi-location brands — direct SOCi competitor. Their Listings AI product is the paid version of the audit you run for free.</t>
+          <t>Conversational AI agents for customer experience, median posted comp around $250K, actively hiring FDEs. Track it. FDE postings grew more than 800% year over year — this function is where technical sales is heading and you want to be qualified before the wave crests.</t>
         </is>
       </c>
       <c r="G28" s="7" t="inlineStr">
         <is>
-          <t>SDR · Solutions · CS</t>
-        </is>
-      </c>
-      <c r="H28" s="9" t="inlineStr">
-        <is>
-          <t>https://birdeye.com/careers/</t>
+          <t>Agent deployment · enterprise CX architecture</t>
+        </is>
+      </c>
+      <c r="H28" s="7" t="inlineStr">
+        <is>
+          <t>Forward Deployed Engineer</t>
+        </is>
+      </c>
+      <c r="I28" s="9" t="inlineStr">
+        <is>
+          <t>https://sierra.ai/careers</t>
         </is>
       </c>
     </row>
     <row r="29" ht="46" customHeight="1">
       <c r="A29" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>Decagon</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>San Francisco</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="F29" s="7" t="inlineStr">
+        <is>
+          <t>AI support agents, ~210 employees, $250M Series D in January 2026, hiring aggressively across engineering and forward-deployed roles.</t>
+        </is>
+      </c>
+      <c r="G29" s="7" t="inlineStr">
+        <is>
+          <t>Agent deployment · post-sale technical ownership</t>
+        </is>
+      </c>
+      <c r="H29" s="7" t="inlineStr">
+        <is>
+          <t>Forward Deployed Engineer · Solutions</t>
+        </is>
+      </c>
+      <c r="I29" s="9" t="inlineStr">
+        <is>
+          <t>https://decagon.ai/careers</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="60" customHeight="1">
+      <c r="A30" s="6" t="n">
         <v>24</v>
       </c>
-      <c r="B29" s="7" t="inlineStr">
-        <is>
-          <t>Podium</t>
-        </is>
-      </c>
-      <c r="C29" s="7" t="inlineStr">
-        <is>
-          <t>Lehi, UT</t>
-        </is>
-      </c>
-      <c r="D29" s="7" t="inlineStr">
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>SF / Remote</t>
+        </is>
+      </c>
+      <c r="D30" s="7" t="inlineStr">
         <is>
           <t>Remote-friendly</t>
         </is>
       </c>
-      <c r="E29" s="8" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="F29" s="7" t="inlineStr">
-        <is>
-          <t>SMS-first SMB platform with an AI Employee product that converts leads rather than just replying to reviews. Same buyer, different wedge.</t>
-        </is>
-      </c>
-      <c r="G29" s="7" t="inlineStr">
-        <is>
-          <t>SDR · AE SMB</t>
-        </is>
-      </c>
-      <c r="H29" s="9" t="inlineStr">
-        <is>
-          <t>https://www.podium.com/careers/</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="46" customHeight="1">
-      <c r="A30" s="6" t="n">
+      <c r="E30" s="10" t="inlineStr">
+        <is>
+          <t>AIM LATER</t>
+        </is>
+      </c>
+      <c r="F30" s="7" t="inlineStr">
+        <is>
+          <t>Honest read: Forward Deployed Engineer, Applied AI is the role your ambition points at, and it pays north of $300K base at senior levels — but it expects deep ML literacy plus production coding and runs a five-stage loop ending in onsite system design. A 3–5 year target. The route there is GTM engineering, then solutions engineering, then this.</t>
+        </is>
+      </c>
+      <c r="G30" s="7" t="inlineStr">
+        <is>
+          <t>(the destination, not the next step)</t>
+        </is>
+      </c>
+      <c r="H30" s="7" t="inlineStr">
+        <is>
+          <t>FDE Applied AI · Solutions Architect</t>
+        </is>
+      </c>
+      <c r="I30" s="9" t="inlineStr">
+        <is>
+          <t>https://www.anthropic.com/careers</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="60" customHeight="1">
+      <c r="A31" s="6" t="n">
         <v>25</v>
       </c>
-      <c r="B30" s="7" t="inlineStr">
-        <is>
-          <t>Yext</t>
-        </is>
-      </c>
-      <c r="C30" s="7" t="inlineStr">
-        <is>
-          <t>New York / Remote</t>
-        </is>
-      </c>
-      <c r="D30" s="7" t="inlineStr">
-        <is>
-          <t>Remote-friendly</t>
-        </is>
-      </c>
-      <c r="E30" s="8" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="F30" s="7" t="inlineStr">
-        <is>
-          <t>The infrastructure underneath much of local search — Semrush white-labels Yext for its listings product. Enterprise-grade citation and listings management. Learning this stack makes your local-SEO claims real.</t>
-        </is>
-      </c>
-      <c r="G30" s="7" t="inlineStr">
-        <is>
-          <t>Solutions Consultant · Sales Engineer</t>
-        </is>
-      </c>
-      <c r="H30" s="9" t="inlineStr">
-        <is>
-          <t>https://www.yext.com/careers</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="46" customHeight="1">
-      <c r="A31" s="6" t="n">
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>SF / Seattle / DC</t>
+        </is>
+      </c>
+      <c r="D31" s="7" t="inlineStr">
+        <is>
+          <t>Hybrid (3 days)</t>
+        </is>
+      </c>
+      <c r="E31" s="10" t="inlineStr">
+        <is>
+          <t>AIM LATER</t>
+        </is>
+      </c>
+      <c r="F31" s="7" t="inlineStr">
+        <is>
+          <t>Same read. FDE reqs want 5–7+ years production full-stack, Python and TypeScript, SQL and Spark, AWS/GCP, Docker and Kubernetes, plus up to 50% travel. Both labs announced billion-dollar FDE pushes within days of each other in May 2026, which is exactly why the bar is where it is.</t>
+        </is>
+      </c>
+      <c r="G31" s="7" t="inlineStr">
+        <is>
+          <t>(the destination, not the next step)</t>
+        </is>
+      </c>
+      <c r="H31" s="7" t="inlineStr">
+        <is>
+          <t>Forward Deployed Software Engineer</t>
+        </is>
+      </c>
+      <c r="I31" s="9" t="inlineStr">
+        <is>
+          <t>https://openai.com/careers/</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="26" customHeight="1">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>LANE 5 — SMB, LOCAL SEARCH &amp; MAIN STREET  ·  the lane where you already have proprietary knowledge. Nobody else applying has cold-called these owners.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="60" customHeight="1">
+      <c r="A33" s="6" t="n">
         <v>26</v>
       </c>
-      <c r="B31" s="7" t="inlineStr">
-        <is>
-          <t>Block (Square)</t>
-        </is>
-      </c>
-      <c r="C31" s="7" t="inlineStr">
-        <is>
-          <t>Multi-city</t>
-        </is>
-      </c>
-      <c r="D31" s="7" t="inlineStr">
-        <is>
-          <t>Varies</t>
-        </is>
-      </c>
-      <c r="E31" s="8" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="F31" s="7" t="inlineStr">
-        <is>
-          <t>Merchant services to small businesses at enormous scale. Currently hiring BDRs in Seattle, NYC, DC and Dublin rather than LA — set an alert and wait for a West Coast wave.</t>
-        </is>
-      </c>
-      <c r="G31" s="7" t="inlineStr">
-        <is>
-          <t>BDR Associate · Account Management</t>
-        </is>
-      </c>
-      <c r="H31" s="9" t="inlineStr">
-        <is>
-          <t>https://block.xyz/careers/jobs</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="22" customHeight="1">
-      <c r="A32" s="4" t="inlineStr">
-        <is>
-          <t>LANE 4 — APPLIED AI &amp; AI ENABLEMENT  ·  aim carefully. Read the reality check at the bottom of this block.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="46" customHeight="1">
-      <c r="A33" s="6" t="n">
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>SOCi</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>San Diego, CA</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t>SoCal / hybrid</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>VERIFIED ACTIVE</t>
+        </is>
+      </c>
+      <c r="F33" s="7" t="inlineStr">
+        <is>
+          <t>Still the single most on-thesis company in the file. 632 employees, and the product is an agentic AI workforce running local search, listings, reviews and social for 1,000+ multi-location brands. Social Hog at enterprise scale, automated. You can recite the pain in their pitch from memory.</t>
+        </is>
+      </c>
+      <c r="G33" s="7" t="inlineStr">
+        <is>
+          <t>Agentic AI applied to local search · multi-location GTM</t>
+        </is>
+      </c>
+      <c r="H33" s="7" t="inlineStr">
+        <is>
+          <t>Solutions Consultant · SDR · CS</t>
+        </is>
+      </c>
+      <c r="I33" s="9" t="inlineStr">
+        <is>
+          <t>https://www.soci.ai/careers/</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="46" customHeight="1">
+      <c r="A34" s="6" t="n">
         <v>27</v>
       </c>
-      <c r="B33" s="7" t="inlineStr">
-        <is>
-          <t>Kyndryl</t>
-        </is>
-      </c>
-      <c r="C33" s="7" t="inlineStr">
-        <is>
-          <t>Remote</t>
-        </is>
-      </c>
-      <c r="D33" s="7" t="inlineStr">
-        <is>
-          <t>Remote</t>
-        </is>
-      </c>
-      <c r="E33" s="8" t="inlineStr">
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>Tebra (Kareo + PatientPop)</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>Newport Beach, CA</t>
+        </is>
+      </c>
+      <c r="D34" s="7" t="inlineStr">
+        <is>
+          <t>SoCal / hybrid</t>
+        </is>
+      </c>
+      <c r="E34" s="8" t="inlineStr">
         <is>
           <t>VERIFIED HIRING</t>
         </is>
       </c>
-      <c r="F33" s="7" t="inlineStr">
-        <is>
-          <t>The most realistic salaried AI-enablement job I could verify anywhere — a live Workday req, not an aspiration. Enterprise AI adoption, change management, training. Apply this week.</t>
-        </is>
-      </c>
-      <c r="G33" s="7" t="inlineStr">
-        <is>
-          <t>AI Enablement Specialist</t>
-        </is>
-      </c>
-      <c r="H33" s="9" t="inlineStr">
-        <is>
-          <t>https://kyndryl.wd5.myworkdayjobs.com/KyndrylProfessionalCareers</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="48" customHeight="1">
-      <c r="A34" s="6" t="n">
-        <v>28</v>
-      </c>
-      <c r="B34" s="7" t="inlineStr">
-        <is>
-          <t>Glean</t>
-        </is>
-      </c>
-      <c r="C34" s="7" t="inlineStr">
-        <is>
-          <t>Remote (US)</t>
-        </is>
-      </c>
-      <c r="D34" s="7" t="inlineStr">
-        <is>
-          <t>Remote</t>
-        </is>
-      </c>
-      <c r="E34" s="8" t="inlineStr">
-        <is>
-          <t>VERIFIED HIRING</t>
-        </is>
-      </c>
       <c r="F34" s="7" t="inlineStr">
         <is>
-          <t>Enterprise AI search and agents, hiring remote US Solutions Engineers at $110K–$235K. The SE role is demos, architecture explanation and proof-of-value exercises — the same shape as your Inbenta work, one generation of technology later. Current reqs are senior; watch for a mid-level or SMB-segment opening.</t>
+          <t>An hour from you, active Greenhouse board. PatientPop sells digital presence, reputation and local visibility to independent practices under 10 providers. Built for Main Street, pointed at doctors.</t>
         </is>
       </c>
       <c r="G34" s="7" t="inlineStr">
         <is>
-          <t>Solutions Engineer</t>
-        </is>
-      </c>
-      <c r="H34" s="9" t="inlineStr">
-        <is>
-          <t>https://www.glean.com/careers</t>
+          <t>Vertical SaaS · healthcare SMB marketing</t>
+        </is>
+      </c>
+      <c r="H34" s="7" t="inlineStr">
+        <is>
+          <t>Solutions Consultant · SDR · CS</t>
+        </is>
+      </c>
+      <c r="I34" s="9" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/tebra</t>
         </is>
       </c>
     </row>
     <row r="35" ht="48" customHeight="1">
       <c r="A35" s="6" t="n">
+        <v>28</v>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>Owner.com</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>Remote-first (SF)</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>VERIFIED HIRING</t>
+        </is>
+      </c>
+      <c r="F35" s="7" t="inlineStr">
+        <is>
+          <t>20,000+ restaurant owners, ~$200M saved in fees, team from Shopify, HubSpot, DoorDash, ServiceTitan and Stripe. Explicitly wants 1–2 years of high-volume SMB SaaS closing — the rare req written AT your level instead of above it.</t>
+        </is>
+      </c>
+      <c r="G35" s="7" t="inlineStr">
+        <is>
+          <t>High-velocity SMB closing · restaurant vertical</t>
+        </is>
+      </c>
+      <c r="H35" s="7" t="inlineStr">
+        <is>
+          <t>AE · Outbound AE · CS Manager</t>
+        </is>
+      </c>
+      <c r="I35" s="9" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="46" customHeight="1">
+      <c r="A36" s="6" t="n">
         <v>29</v>
       </c>
-      <c r="B35" s="7" t="inlineStr">
-        <is>
-          <t>Scale AI</t>
-        </is>
-      </c>
-      <c r="C35" s="7" t="inlineStr">
-        <is>
-          <t>San Francisco</t>
-        </is>
-      </c>
-      <c r="D35" s="7" t="inlineStr">
-        <is>
-          <t>Remote-friendly</t>
-        </is>
-      </c>
-      <c r="E35" s="8" t="inlineStr">
-        <is>
-          <t>ACTIVE — PIVOTED</t>
-        </is>
-      </c>
-      <c r="F35" s="7" t="inlineStr">
-        <is>
-          <t>Worth targeting, but on the commercial side. They cut 200 FTEs and 500 contractors after the Meta deal and flipped from 70% data labeling to an apps business now at ~$200M annualized, with plans to add ~500 people. Chase the apps and GTM roles, not the annotation queue.</t>
-        </is>
-      </c>
-      <c r="G35" s="7" t="inlineStr">
-        <is>
-          <t>GTM · Solutions · Deployment</t>
-        </is>
-      </c>
-      <c r="H35" s="9" t="inlineStr">
-        <is>
-          <t>https://scale.com/careers</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="48" customHeight="1">
-      <c r="A36" s="6" t="n">
-        <v>30</v>
-      </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>Sierra AI</t>
+          <t>Housecall Pro</t>
         </is>
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>San Francisco</t>
+          <t>San Diego, CA</t>
         </is>
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>Hybrid</t>
+          <t>Remote-first</t>
         </is>
       </c>
       <c r="E36" s="8" t="inlineStr">
         <is>
-          <t>ACTIVE</t>
+          <t>VERIFIED HIRING</t>
         </is>
       </c>
       <c r="F36" s="7" t="inlineStr">
         <is>
-          <t>Conversational AI agents for customer experience, hiring forward-deployed engineers, median posted comp around $250K. Aspirational rather than immediate — but a company to track, because the FDE function is where technical sales is heading.</t>
+          <t>Genuinely remote-first, currently posting a remote US Inside Sales Rep. Sells to plumbers, electricians and HVAC contractors — the precise owner profile you already dial.</t>
         </is>
       </c>
       <c r="G36" s="7" t="inlineStr">
         <is>
-          <t>Forward Deployed Engineer</t>
-        </is>
-      </c>
-      <c r="H36" s="9" t="inlineStr">
-        <is>
-          <t>https://sierra.ai/careers</t>
+          <t>Home-services vertical · inside sales at volume</t>
+        </is>
+      </c>
+      <c r="H36" s="7" t="inlineStr">
+        <is>
+          <t>Inside Sales · CS · Sales Training</t>
+        </is>
+      </c>
+      <c r="I36" s="9" t="inlineStr">
+        <is>
+          <t>https://www.housecallpro.com/careers/</t>
         </is>
       </c>
     </row>
     <row r="37" ht="46" customHeight="1">
       <c r="A37" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>ServiceTitan</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>Glendale, CA</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="inlineStr">
+        <is>
+          <t>LA — hybrid</t>
+        </is>
+      </c>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>VERIFIED HIRING</t>
+        </is>
+      </c>
+      <c r="F37" s="7" t="inlineStr">
+        <is>
+          <t>The largest home-services software company in the country, in Glendale. Also the most credible LA launchpad here — ex-ServiceTitan people turn up on founding teams like Owner.com's.</t>
+        </is>
+      </c>
+      <c r="G37" s="7" t="inlineStr">
+        <is>
+          <t>Vertical SaaS at scale · LA network</t>
+        </is>
+      </c>
+      <c r="H37" s="7" t="inlineStr">
+        <is>
+          <t>SDR · Solutions Consultant · CS</t>
+        </is>
+      </c>
+      <c r="I37" s="9" t="inlineStr">
+        <is>
+          <t>https://www.servicetitan.com/careers</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="46" customHeight="1">
+      <c r="A38" s="6" t="n">
         <v>31</v>
       </c>
-      <c r="B37" s="7" t="inlineStr">
-        <is>
-          <t>Decagon</t>
-        </is>
-      </c>
-      <c r="C37" s="7" t="inlineStr">
-        <is>
-          <t>San Francisco</t>
-        </is>
-      </c>
-      <c r="D37" s="7" t="inlineStr">
-        <is>
-          <t>Hybrid</t>
-        </is>
-      </c>
-      <c r="E37" s="8" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="F37" s="7" t="inlineStr">
-        <is>
-          <t>AI support agents, ~210 employees, $250M Series D in January 2026 and hiring aggressively across engineering and forward-deployed roles. Same note as Sierra: track it, build toward it.</t>
-        </is>
-      </c>
-      <c r="G37" s="7" t="inlineStr">
-        <is>
-          <t>Forward Deployed Engineer · Solutions</t>
-        </is>
-      </c>
-      <c r="H37" s="9" t="inlineStr">
-        <is>
-          <t>https://decagon.ai/careers</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="72" customHeight="1">
-      <c r="A38" s="6" t="n">
+      <c r="B38" s="7" t="inlineStr">
+        <is>
+          <t>Otter (CloudKitchens)</t>
+        </is>
+      </c>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>Los Angeles, CA</t>
+        </is>
+      </c>
+      <c r="D38" s="7" t="inlineStr">
+        <is>
+          <t>LA — on-site</t>
+        </is>
+      </c>
+      <c r="E38" s="8" t="inlineStr">
+        <is>
+          <t>VERIFIED HIRING</t>
+        </is>
+      </c>
+      <c r="F38" s="7" t="inlineStr">
+        <is>
+          <t>Solutions Engineer open right now on their own Greenhouse board, in LA, explicitly no cold calls. Still your best single application in this file.</t>
+        </is>
+      </c>
+      <c r="G38" s="7" t="inlineStr">
+        <is>
+          <t>Pre-sales engineering · POS deployment</t>
+        </is>
+      </c>
+      <c r="H38" s="7" t="inlineStr">
+        <is>
+          <t>Solutions Engineer · Implementation</t>
+        </is>
+      </c>
+      <c r="I38" s="9" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/otter</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="46" customHeight="1">
+      <c r="A39" s="6" t="n">
         <v>32</v>
       </c>
-      <c r="B38" s="7" t="inlineStr">
-        <is>
-          <t>Anthropic</t>
-        </is>
-      </c>
-      <c r="C38" s="7" t="inlineStr">
-        <is>
-          <t>SF / Remote</t>
-        </is>
-      </c>
-      <c r="D38" s="7" t="inlineStr">
-        <is>
-          <t>Remote-friendly</t>
-        </is>
-      </c>
-      <c r="E38" s="8" t="inlineStr">
-        <is>
-          <t>ACTIVE — AIM LATER</t>
-        </is>
-      </c>
-      <c r="F38" s="7" t="inlineStr">
-        <is>
-          <t>REALITY CHECK, and I would rather you hear it from me than from a rejection email. Forward Deployed Engineer, Applied AI is real and it is the role that fits your ambition — but it pays north of $300K base at senior levels, expects deep ML literacy plus production coding, and runs a five-stage loop ending in onsite system design. It is a 3–5 year target, not an August application. Build toward it through GTM engineering and solutions work.</t>
-        </is>
-      </c>
-      <c r="G38" s="7" t="inlineStr">
-        <is>
-          <t>FDE Applied AI · Solutions Architect</t>
-        </is>
-      </c>
-      <c r="H38" s="9" t="inlineStr">
-        <is>
-          <t>https://www.anthropic.com/careers</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="60" customHeight="1">
-      <c r="A39" s="6" t="n">
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>Boulevard</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>Los Angeles, CA</t>
+        </is>
+      </c>
+      <c r="D39" s="7" t="inlineStr">
+        <is>
+          <t>LA — hybrid</t>
+        </is>
+      </c>
+      <c r="E39" s="8" t="inlineStr">
+        <is>
+          <t>VERIFIED HIRING</t>
+        </is>
+      </c>
+      <c r="F39" s="7" t="inlineStr">
+        <is>
+          <t>LA HQ, ~260 people, selling to salons, spas and med-spas on Salesforce and Outreach. Local, venture-backed, and the buyer is one you have already sat across from.</t>
+        </is>
+      </c>
+      <c r="G39" s="7" t="inlineStr">
+        <is>
+          <t>Appointment-based SMB vertical</t>
+        </is>
+      </c>
+      <c r="H39" s="7" t="inlineStr">
+        <is>
+          <t>SDR · CS · Solutions</t>
+        </is>
+      </c>
+      <c r="I39" s="9" t="inlineStr">
+        <is>
+          <t>https://www.joinblvd.com/careers</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="46" customHeight="1">
+      <c r="A40" s="6" t="n">
         <v>33</v>
       </c>
-      <c r="B39" s="7" t="inlineStr">
-        <is>
-          <t>OpenAI</t>
-        </is>
-      </c>
-      <c r="C39" s="7" t="inlineStr">
-        <is>
-          <t>SF / Seattle / DC</t>
-        </is>
-      </c>
-      <c r="D39" s="7" t="inlineStr">
-        <is>
-          <t>Hybrid (3 days)</t>
-        </is>
-      </c>
-      <c r="E39" s="8" t="inlineStr">
-        <is>
-          <t>ACTIVE — AIM LATER</t>
-        </is>
-      </c>
-      <c r="F39" s="7" t="inlineStr">
-        <is>
-          <t>Same reality check. Their FDE postings ask for 5–7+ years of production full-stack engineering, Python and TypeScript, SQL and Spark, AWS/GCP, Docker and Kubernetes, plus up to 50% travel. Both labs announced billion-dollar FDE pushes in May 2026, which is exactly why the bar is high. Track it, do not apply yet.</t>
-        </is>
-      </c>
-      <c r="G39" s="7" t="inlineStr">
-        <is>
-          <t>Forward Deployed Software Engineer</t>
-        </is>
-      </c>
-      <c r="H39" s="9" t="inlineStr">
-        <is>
-          <t>https://openai.com/careers/</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="22" customHeight="1">
-      <c r="A40" s="4" t="inlineStr">
-        <is>
-          <t>LANE 5 — LA COMPANIES WORTH WANTING  ·  local, growing, and hiring on the commercial side.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="48" customHeight="1">
+      <c r="B40" s="7" t="inlineStr">
+        <is>
+          <t>Yelp</t>
+        </is>
+      </c>
+      <c r="C40" s="7" t="inlineStr">
+        <is>
+          <t>Remote-first</t>
+        </is>
+      </c>
+      <c r="D40" s="7" t="inlineStr">
+        <is>
+          <t>Remote (West)</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="inlineStr">
+        <is>
+          <t>VERIFIED HIRING</t>
+        </is>
+      </c>
+      <c r="F40" s="7" t="inlineStr">
+        <is>
+          <t>90%+ of openings remote, Western US residency required for the inside sales role — LA qualifies. Local search is the entire company.</t>
+        </is>
+      </c>
+      <c r="G40" s="7" t="inlineStr">
+        <is>
+          <t>Local search economics · SMB advertising</t>
+        </is>
+      </c>
+      <c r="H40" s="7" t="inlineStr">
+        <is>
+          <t>Inside Sales · Local AE</t>
+        </is>
+      </c>
+      <c r="I40" s="9" t="inlineStr">
+        <is>
+          <t>https://www.yelp.careers/us/en</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="46" customHeight="1">
       <c r="A41" s="6" t="n">
         <v>34</v>
       </c>
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>Whatnot</t>
+          <t>Birdeye</t>
         </is>
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>Los Angeles, CA</t>
+          <t>Palo Alto, CA</t>
         </is>
       </c>
       <c r="D41" s="7" t="inlineStr">
         <is>
-          <t>LA — hybrid</t>
+          <t>Remote-friendly</t>
         </is>
       </c>
       <c r="E41" s="8" t="inlineStr">
         <is>
-          <t>VERIFIED HIRING</t>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="F41" s="7" t="inlineStr">
         <is>
-          <t>LA-headquartered livestream shopping, ~$12B valuation, headcount up 31% last year, ~1,200 employees and 9 openings near LA. They require you to live within commuting distance of the LA, NYC or SF hub — you already do. One of the few genuinely fast-growing large LA tech companies.</t>
+          <t>Reviews, listings and messaging AI for multi-location brands — SOCi's direct competitor. Their Listings AI is the paid version of the audit you run for free.</t>
         </is>
       </c>
       <c r="G41" s="7" t="inlineStr">
         <is>
-          <t>GTM · Partnerships · Category</t>
-        </is>
-      </c>
-      <c r="H41" s="9" t="inlineStr">
-        <is>
-          <t>https://careers.whatnot.com/</t>
+          <t>Reputation and listings stack</t>
+        </is>
+      </c>
+      <c r="H41" s="7" t="inlineStr">
+        <is>
+          <t>SDR · Solutions · CS</t>
+        </is>
+      </c>
+      <c r="I41" s="9" t="inlineStr">
+        <is>
+          <t>https://birdeye.com/careers/</t>
         </is>
       </c>
     </row>
@@ -4120,204 +4296,229 @@
       </c>
       <c r="B42" s="7" t="inlineStr">
         <is>
-          <t>GoodRx</t>
+          <t>Yext</t>
         </is>
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>Santa Monica, CA</t>
+          <t>New York / Remote</t>
         </is>
       </c>
       <c r="D42" s="7" t="inlineStr">
         <is>
-          <t>LA — hybrid</t>
+          <t>Remote-friendly</t>
         </is>
       </c>
       <c r="E42" s="8" t="inlineStr">
         <is>
-          <t>VERIFIED HIRING</t>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="F42" s="7" t="inlineStr">
         <is>
-          <t>Santa Monica HQ with ~15 open roles spanning Marketing, Data &amp; Analytics, Sales, and AI/ML. Consumer healthcare pricing — decision-making under confusion and cost pressure, which is a theme you already think about.</t>
+          <t>The infrastructure under much of local search — Semrush white-labels Yext for listings. Learning this stack makes your local-SEO claims verifiable rather than assertable.</t>
         </is>
       </c>
       <c r="G42" s="7" t="inlineStr">
         <is>
-          <t>Sales · Marketing · Analytics</t>
-        </is>
-      </c>
-      <c r="H42" s="9" t="inlineStr">
-        <is>
-          <t>https://www.goodrx.com/jobs</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="46" customHeight="1">
-      <c r="A43" s="6" t="n">
-        <v>36</v>
-      </c>
-      <c r="B43" s="7" t="inlineStr">
-        <is>
-          <t>Artera</t>
-        </is>
-      </c>
-      <c r="C43" s="7" t="inlineStr">
-        <is>
-          <t>Santa Barbara + LA</t>
-        </is>
-      </c>
-      <c r="D43" s="7" t="inlineStr">
-        <is>
-          <t>SoCal — hybrid</t>
-        </is>
-      </c>
-      <c r="E43" s="8" t="inlineStr">
-        <is>
-          <t>VERIFIED HIRING</t>
-        </is>
-      </c>
-      <c r="F43" s="7" t="inlineStr">
-        <is>
-          <t>Agentic AI voice and text for patient communication, ~11 openings, hybrid three days a week, hires in the LA area. Real applied-AI work at a company small enough that a generalist who can sell and build is obviously useful.</t>
-        </is>
-      </c>
-      <c r="G43" s="7" t="inlineStr">
-        <is>
-          <t>Account Executive · Solutions</t>
-        </is>
-      </c>
-      <c r="H43" s="9" t="inlineStr">
-        <is>
-          <t>https://artera.io/careers</t>
+          <t>Enterprise listings and citation infrastructure</t>
+        </is>
+      </c>
+      <c r="H42" s="7" t="inlineStr">
+        <is>
+          <t>Solutions Consultant · Sales Engineer</t>
+        </is>
+      </c>
+      <c r="I42" s="9" t="inlineStr">
+        <is>
+          <t>https://www.yext.com/careers</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="39" customHeight="1">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>LANE 6 — THINGS YOU ACTUALLY CARE ABOUT  ·  new in v2. You listed chess, drums, fitness, content and behavior change as your interests. These are real employers in exactly those categories, and caring about the product is not a soft factor — it is the difference between a good interview and a great one.</t>
         </is>
       </c>
     </row>
     <row r="44" ht="46" customHeight="1">
       <c r="A44" s="6" t="n">
+        <v>36</v>
+      </c>
+      <c r="B44" s="7" t="inlineStr">
+        <is>
+          <t>Chess.com</t>
+        </is>
+      </c>
+      <c r="C44" s="7" t="inlineStr">
+        <is>
+          <t>Fully remote</t>
+        </is>
+      </c>
+      <c r="D44" s="7" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="E44" s="8" t="inlineStr">
+        <is>
+          <t>VERIFIED HIRING</t>
+        </is>
+      </c>
+      <c r="F44" s="7" t="inlineStr">
+        <is>
+          <t>250 million players, 600+ people across 60 countries, fully remote, 19 open roles. You play chess. This is not a stretch of a story — it is the easiest authentic 'why us' you will ever write.</t>
+        </is>
+      </c>
+      <c r="G44" s="7" t="inlineStr">
+        <is>
+          <t>Consumer product at massive scale · fully-distributed work</t>
+        </is>
+      </c>
+      <c r="H44" s="7" t="inlineStr">
+        <is>
+          <t>Growth · Partnerships · Analytics</t>
+        </is>
+      </c>
+      <c r="I44" s="9" t="inlineStr">
+        <is>
+          <t>https://www.chess.com/jobs</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="60" customHeight="1">
+      <c r="A45" s="6" t="n">
         <v>37</v>
       </c>
-      <c r="B44" s="7" t="inlineStr">
-        <is>
-          <t>Anduril</t>
-        </is>
-      </c>
-      <c r="C44" s="7" t="inlineStr">
-        <is>
-          <t>Costa Mesa, CA</t>
-        </is>
-      </c>
-      <c r="D44" s="7" t="inlineStr">
-        <is>
-          <t>OC — on-site</t>
-        </is>
-      </c>
-      <c r="E44" s="8" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="F44" s="7" t="inlineStr">
-        <is>
-          <t>Large, growing, and hires heavily on the commercial and program side, not only engineering. Roughly an hour from you. Worth a look if you want scale and intensity.</t>
-        </is>
-      </c>
-      <c r="G44" s="7" t="inlineStr">
-        <is>
-          <t>Business Development · Solutions</t>
-        </is>
-      </c>
-      <c r="H44" s="9" t="inlineStr">
-        <is>
-          <t>https://www.anduril.com/careers/</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="46" customHeight="1">
-      <c r="A45" s="6" t="n">
-        <v>38</v>
-      </c>
       <c r="B45" s="7" t="inlineStr">
         <is>
-          <t>Scopely</t>
+          <t>WHOOP</t>
         </is>
       </c>
       <c r="C45" s="7" t="inlineStr">
         <is>
-          <t>Culver City, CA</t>
+          <t>Boston, MA</t>
         </is>
       </c>
       <c r="D45" s="7" t="inlineStr">
         <is>
-          <t>LA — hybrid</t>
+          <t>Hybrid / some remote</t>
         </is>
       </c>
       <c r="E45" s="8" t="inlineStr">
         <is>
-          <t>ACTIVE</t>
+          <t>VERIFIED HIRING</t>
         </is>
       </c>
       <c r="F45" s="7" t="inlineStr">
         <is>
-          <t>One of the biggest LA tech employers, mobile games at real scale. Less thesis-aligned, more about compensation, stability and staying in the LA network.</t>
+          <t>Announced a 2026 surge of 600+ new roles across technical, scientific, creative and commercial functions. Their Journal feature recommends behaviors to add or remove based on your own data — that is behavior change as a product, which is on your stated interest list. Boston-weighted, so filter for remote.</t>
         </is>
       </c>
       <c r="G45" s="7" t="inlineStr">
         <is>
-          <t>Partnerships · BD · Analytics</t>
-        </is>
-      </c>
-      <c r="H45" s="9" t="inlineStr">
-        <is>
-          <t>https://scopely.com/careers/</t>
+          <t>Behavior-change product mechanics · wearables GTM</t>
+        </is>
+      </c>
+      <c r="H45" s="7" t="inlineStr">
+        <is>
+          <t>Commercial · Enablement · Partnerships</t>
+        </is>
+      </c>
+      <c r="I45" s="9" t="inlineStr">
+        <is>
+          <t>https://www.whoop.com/careers/</t>
         </is>
       </c>
     </row>
     <row r="46" ht="46" customHeight="1">
       <c r="A46" s="6" t="n">
+        <v>38</v>
+      </c>
+      <c r="B46" s="7" t="inlineStr">
+        <is>
+          <t>Oura</t>
+        </is>
+      </c>
+      <c r="C46" s="7" t="inlineStr">
+        <is>
+          <t>SF / Remote</t>
+        </is>
+      </c>
+      <c r="D46" s="7" t="inlineStr">
+        <is>
+          <t>Remote-friendly</t>
+        </is>
+      </c>
+      <c r="E46" s="8" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="F46" s="7" t="inlineStr">
+        <is>
+          <t>Hiring a Director of Commercial Enablement focused on B2B sales enablement — the exact function, in the exact category you care about. That specific req is senior, but it tells you they build enablement teams.</t>
+        </is>
+      </c>
+      <c r="G46" s="7" t="inlineStr">
+        <is>
+          <t>Sales enablement inside a health-behavior company</t>
+        </is>
+      </c>
+      <c r="H46" s="7" t="inlineStr">
+        <is>
+          <t>Commercial Enablement · Partnerships</t>
+        </is>
+      </c>
+      <c r="I46" s="9" t="inlineStr">
+        <is>
+          <t>https://ouraring.com/careers</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="46" customHeight="1">
+      <c r="A47" s="6" t="n">
         <v>39</v>
       </c>
-      <c r="B46" s="7" t="inlineStr">
-        <is>
-          <t>FloQast</t>
-        </is>
-      </c>
-      <c r="C46" s="7" t="inlineStr">
-        <is>
-          <t>Burbank, CA</t>
-        </is>
-      </c>
-      <c r="D46" s="7" t="inlineStr">
-        <is>
-          <t>LA — hybrid</t>
-        </is>
-      </c>
-      <c r="E46" s="8" t="inlineStr">
+      <c r="B47" s="7" t="inlineStr">
+        <is>
+          <t>Hinge Health</t>
+        </is>
+      </c>
+      <c r="C47" s="7" t="inlineStr">
+        <is>
+          <t>SF / Remote</t>
+        </is>
+      </c>
+      <c r="D47" s="7" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="E47" s="8" t="inlineStr">
         <is>
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="F46" s="7" t="inlineStr">
-        <is>
-          <t>Accounting workflow automation, Burbank-based, consistently strong on LA best-places-to-work lists. Workflow automation sold to finance teams — closer to your AI-workflow lane than it first looks.</t>
-        </is>
-      </c>
-      <c r="G46" s="7" t="inlineStr">
-        <is>
-          <t>SDR · Solutions Consultant · CS</t>
-        </is>
-      </c>
-      <c r="H46" s="9" t="inlineStr">
-        <is>
-          <t>https://floqast.com/careers/</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="22" customHeight="1">
-      <c r="A47" s="4" t="inlineStr">
-        <is>
-          <t>DO NOT BOTHER — verified reasons to skip</t>
+      <c r="F47" s="7" t="inlineStr">
+        <is>
+          <t>Remote sales-enablement roles posted at $84K–$166K depending on location tier. Digital physical therapy — measurable behavior change, enterprise buyers.</t>
+        </is>
+      </c>
+      <c r="G47" s="7" t="inlineStr">
+        <is>
+          <t>Healthcare enablement · payer/employer GTM</t>
+        </is>
+      </c>
+      <c r="H47" s="7" t="inlineStr">
+        <is>
+          <t>Sales Enablement · Partnerships</t>
+        </is>
+      </c>
+      <c r="I47" s="9" t="inlineStr">
+        <is>
+          <t>https://www.hingehealth.com/careers/</t>
         </is>
       </c>
     </row>
@@ -4327,37 +4528,42 @@
       </c>
       <c r="B48" s="7" t="inlineStr">
         <is>
-          <t>BetterUp</t>
+          <t>HeyGen</t>
         </is>
       </c>
       <c r="C48" s="7" t="inlineStr">
         <is>
-          <t>SF / Remote</t>
+          <t>Los Angeles, CA</t>
         </is>
       </c>
       <c r="D48" s="7" t="inlineStr">
         <is>
-          <t>Remote</t>
-        </is>
-      </c>
-      <c r="E48" s="11" t="inlineStr">
-        <is>
-          <t>AVOID</t>
+          <t>LA</t>
+        </is>
+      </c>
+      <c r="E48" s="8" t="inlineStr">
+        <is>
+          <t>VERIFIED HIRING</t>
         </is>
       </c>
       <c r="F48" s="7" t="inlineStr">
         <is>
-          <t>Looks perfect on paper for you — coaching, behavior change, career development. It is not. They laid off ~100 people, missed financial targets, and their coaches revolted over pay cuts. Employee reviews describe constant strategy shifts and moving goalposts. Your coaching certificate deserves a healthier home.</t>
+          <t>LA-headquartered AI video, 150 employees and 94 open positions, 100,000+ businesses using it. AI plus content plus Los Angeles in one company. If you want to be near AI disruption while staying home, this is the most obvious building in the city.</t>
         </is>
       </c>
       <c r="G48" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>AI content tooling · creator and enterprise GTM</t>
         </is>
       </c>
       <c r="H48" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>GTM · Solutions · Partnerships</t>
+        </is>
+      </c>
+      <c r="I48" s="9" t="inlineStr">
+        <is>
+          <t>https://www.heygen.com/careers</t>
         </is>
       </c>
     </row>
@@ -4367,37 +4573,42 @@
       </c>
       <c r="B49" s="7" t="inlineStr">
         <is>
-          <t>Hired.com</t>
+          <t>OpusClip</t>
         </is>
       </c>
       <c r="C49" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Mountain View</t>
         </is>
       </c>
       <c r="D49" s="7" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E49" s="11" t="inlineStr">
-        <is>
-          <t>DEAD</t>
+          <t>Remote-friendly</t>
+        </is>
+      </c>
+      <c r="E49" s="8" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="F49" s="7" t="inlineStr">
         <is>
-          <t>Shut down June 2024. Included here only so it does not reappear in a future list.</t>
+          <t>10M+ creators and businesses in 18 months, ~100 people. The content-repurposing layer you already think about when you plan your own posting.</t>
         </is>
       </c>
       <c r="G49" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Creator-economy GTM · viral product loops</t>
         </is>
       </c>
       <c r="H49" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>GTM · Partnerships</t>
+        </is>
+      </c>
+      <c r="I49" s="9" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/opusclip</t>
         </is>
       </c>
     </row>
@@ -4407,12 +4618,12 @@
       </c>
       <c r="B50" s="7" t="inlineStr">
         <is>
-          <t>Skyray Ventures</t>
+          <t>Splice</t>
         </is>
       </c>
       <c r="C50" s="7" t="inlineStr">
         <is>
-          <t>Lahore, PK</t>
+          <t>Remote (US/UK)</t>
         </is>
       </c>
       <c r="D50" s="7" t="inlineStr">
@@ -4420,24 +4631,29 @@
           <t>Remote</t>
         </is>
       </c>
-      <c r="E50" s="11" t="inlineStr">
-        <is>
-          <t>AVOID</t>
+      <c r="E50" s="8" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="F50" s="7" t="inlineStr">
         <is>
-          <t>Reviews titled 'Fake Promises'; consistent reports of low pay and micromanagement.</t>
+          <t>Music production platform — samples, AI tools and affordable DAWs — with a remote culture and 8 open roles on Greenhouse. You play drums. Small company, low opening volume, but worth a standing alert.</t>
         </is>
       </c>
       <c r="G50" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Creator subscription economics</t>
         </is>
       </c>
       <c r="H50" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>GTM · Partnerships</t>
+        </is>
+      </c>
+      <c r="I50" s="9" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/splice</t>
         </is>
       </c>
     </row>
@@ -4447,100 +4663,623 @@
       </c>
       <c r="B51" s="7" t="inlineStr">
         <is>
+          <t>Snap</t>
+        </is>
+      </c>
+      <c r="C51" s="7" t="inlineStr">
+        <is>
+          <t>Santa Monica, CA</t>
+        </is>
+      </c>
+      <c r="D51" s="7" t="inlineStr">
+        <is>
+          <t>LA — hybrid</t>
+        </is>
+      </c>
+      <c r="E51" s="8" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="F51" s="7" t="inlineStr">
+        <is>
+          <t>Silicon Beach, and moving from filters into foundational AI with generative AI roles paying up to $259,000. The largest concentration of AI work you can reach without leaving LA County.</t>
+        </is>
+      </c>
+      <c r="G51" s="7" t="inlineStr">
+        <is>
+          <t>Consumer AI at scale · LA network density</t>
+        </is>
+      </c>
+      <c r="H51" s="7" t="inlineStr">
+        <is>
+          <t>Partnerships · Commercial</t>
+        </is>
+      </c>
+      <c r="I51" s="9" t="inlineStr">
+        <is>
+          <t>https://careers.snap.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="46" customHeight="1">
+      <c r="A52" s="6" t="n">
+        <v>44</v>
+      </c>
+      <c r="B52" s="7" t="inlineStr">
+        <is>
+          <t>GumGum</t>
+        </is>
+      </c>
+      <c r="C52" s="7" t="inlineStr">
+        <is>
+          <t>Santa Monica, CA</t>
+        </is>
+      </c>
+      <c r="D52" s="7" t="inlineStr">
+        <is>
+          <t>LA — hybrid</t>
+        </is>
+      </c>
+      <c r="E52" s="8" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="F52" s="7" t="inlineStr">
+        <is>
+          <t>Contextual advertising and computer vision, Santa Monica. Placing ads intelligently without personal data — a genuinely interesting constraint, and a mid-size LA company where a generalist gets real scope.</t>
+        </is>
+      </c>
+      <c r="G52" s="7" t="inlineStr">
+        <is>
+          <t>Applied computer vision · adtech GTM</t>
+        </is>
+      </c>
+      <c r="H52" s="7" t="inlineStr">
+        <is>
+          <t>Solutions · Account Management</t>
+        </is>
+      </c>
+      <c r="I52" s="9" t="inlineStr">
+        <is>
+          <t>https://gumgum.com/careers</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="26" customHeight="1">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>DEMOTED FROM v1 — good companies, but you were right that they do not belong. Kept visible so you can see the reasoning rather than wonder where they went.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="46" customHeight="1">
+      <c r="A54" s="6" t="n">
+        <v>45</v>
+      </c>
+      <c r="B54" s="7" t="inlineStr">
+        <is>
+          <t>Scopely</t>
+        </is>
+      </c>
+      <c r="C54" s="7" t="inlineStr">
+        <is>
+          <t>Culver City, CA</t>
+        </is>
+      </c>
+      <c r="D54" s="7" t="inlineStr">
+        <is>
+          <t>LA — hybrid</t>
+        </is>
+      </c>
+      <c r="E54" s="11" t="inlineStr">
+        <is>
+          <t>CUT — NO RAMP</t>
+        </is>
+      </c>
+      <c r="F54" s="7" t="inlineStr">
+        <is>
+          <t>Big LA employer, mobile games. Nothing about it compounds your AI, labor-market or SMB knowledge. It was on the v1 list for LA proximity alone, which is not a good enough reason.</t>
+        </is>
+      </c>
+      <c r="G54" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H54" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I54" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="46" customHeight="1">
+      <c r="A55" s="6" t="n">
+        <v>46</v>
+      </c>
+      <c r="B55" s="7" t="inlineStr">
+        <is>
+          <t>FloQast</t>
+        </is>
+      </c>
+      <c r="C55" s="7" t="inlineStr">
+        <is>
+          <t>Burbank, CA</t>
+        </is>
+      </c>
+      <c r="D55" s="7" t="inlineStr">
+        <is>
+          <t>LA — hybrid</t>
+        </is>
+      </c>
+      <c r="E55" s="11" t="inlineStr">
+        <is>
+          <t>CUT — WEAK FIT</t>
+        </is>
+      </c>
+      <c r="F55" s="7" t="inlineStr">
+        <is>
+          <t>Accounting workflow automation. I argued it was workflow-adjacent. On reflection that is a stretch — the buyer is a controller and the domain teaches you accounting close cycles, not your field.</t>
+        </is>
+      </c>
+      <c r="G55" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H55" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I55" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="46" customHeight="1">
+      <c r="A56" s="6" t="n">
+        <v>47</v>
+      </c>
+      <c r="B56" s="7" t="inlineStr">
+        <is>
+          <t>Anduril</t>
+        </is>
+      </c>
+      <c r="C56" s="7" t="inlineStr">
+        <is>
+          <t>Costa Mesa, CA</t>
+        </is>
+      </c>
+      <c r="D56" s="7" t="inlineStr">
+        <is>
+          <t>OC — on-site</t>
+        </is>
+      </c>
+      <c r="E56" s="11" t="inlineStr">
+        <is>
+          <t>CUT — WRONG FIELD</t>
+        </is>
+      </c>
+      <c r="F56" s="7" t="inlineStr">
+        <is>
+          <t>Excellent company, genuinely hiring, entirely orthogonal to everything you are building. Defense procurement is a different universe from career intelligence.</t>
+        </is>
+      </c>
+      <c r="G56" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H56" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I56" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="46" customHeight="1">
+      <c r="A57" s="6" t="n">
+        <v>48</v>
+      </c>
+      <c r="B57" s="7" t="inlineStr">
+        <is>
+          <t>Block (Square)</t>
+        </is>
+      </c>
+      <c r="C57" s="7" t="inlineStr">
+        <is>
+          <t>Multi-city</t>
+        </is>
+      </c>
+      <c r="D57" s="7" t="inlineStr">
+        <is>
+          <t>Not LA</t>
+        </is>
+      </c>
+      <c r="E57" s="11" t="inlineStr">
+        <is>
+          <t>CUT — LOCATION</t>
+        </is>
+      </c>
+      <c r="F57" s="7" t="inlineStr">
+        <is>
+          <t>SMB merchant services is thesis-aligned, but the open BDR reqs are Seattle, NYC, DC and Dublin. Keep an alert, do not spend application time.</t>
+        </is>
+      </c>
+      <c r="G57" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H57" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I57" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="46" customHeight="1">
+      <c r="A58" s="6" t="n">
+        <v>49</v>
+      </c>
+      <c r="B58" s="7" t="inlineStr">
+        <is>
+          <t>Lightcast</t>
+        </is>
+      </c>
+      <c r="C58" s="7" t="inlineStr">
+        <is>
+          <t>Remote-first</t>
+        </is>
+      </c>
+      <c r="D58" s="7" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="E58" s="10" t="inlineStr">
+        <is>
+          <t>DEMOTED — SLOW</t>
+        </is>
+      </c>
+      <c r="F58" s="7" t="inlineStr">
+        <is>
+          <t>Real labor-market intelligence and a legitimate fit on paper, but it is the incumbent: slower, more enterprise, fewer openings, less learning per month than Mercor, Juicebox or Revelio.</t>
+        </is>
+      </c>
+      <c r="G58" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H58" s="7" t="inlineStr">
+        <is>
+          <t>Solutions Consultant</t>
+        </is>
+      </c>
+      <c r="I58" s="9" t="inlineStr">
+        <is>
+          <t>https://lightcast.io/about/careers</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="48" customHeight="1">
+      <c r="A59" s="6" t="n">
+        <v>50</v>
+      </c>
+      <c r="B59" s="7" t="inlineStr">
+        <is>
+          <t>Eightfold AI / Teal / GoodRx / Artera / Whatnot</t>
+        </is>
+      </c>
+      <c r="C59" s="7" t="inlineStr">
+        <is>
+          <t>Various</t>
+        </is>
+      </c>
+      <c r="D59" s="7" t="inlineStr">
+        <is>
+          <t>Various</t>
+        </is>
+      </c>
+      <c r="E59" s="10" t="inlineStr">
+        <is>
+          <t>DEMOTED — SECOND TIER</t>
+        </is>
+      </c>
+      <c r="F59" s="7" t="inlineStr">
+        <is>
+          <t>All real, all still worth an alert, none worth a slot in your first twenty applications. Eightfold and Teal are fine but low-volume; GoodRx, Artera and Whatnot are good LA employers whose domains do not compound anything you are building.</t>
+        </is>
+      </c>
+      <c r="G59" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H59" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I59" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="22" customHeight="1">
+      <c r="A60" s="4" t="inlineStr">
+        <is>
+          <t>DO NOT BOTHER — verified reasons to skip</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="60" customHeight="1">
+      <c r="A61" s="6" t="n">
+        <v>51</v>
+      </c>
+      <c r="B61" s="7" t="inlineStr">
+        <is>
+          <t>BetterUp</t>
+        </is>
+      </c>
+      <c r="C61" s="7" t="inlineStr">
+        <is>
+          <t>SF / Remote</t>
+        </is>
+      </c>
+      <c r="D61" s="7" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="E61" s="11" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+      <c r="F61" s="7" t="inlineStr">
+        <is>
+          <t>Looks tailor-made for you — coaching, behavior change, career development. It is not. ~100 laid off, missed financial targets, coaches in revolt over pay cuts, and reviews describing constant strategy shifts and moving goalposts. Your coaching certificate deserves a healthier home.</t>
+        </is>
+      </c>
+      <c r="G61" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H61" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I61" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="46" customHeight="1">
+      <c r="A62" s="6" t="n">
+        <v>52</v>
+      </c>
+      <c r="B62" s="7" t="inlineStr">
+        <is>
+          <t>Hired.com</t>
+        </is>
+      </c>
+      <c r="C62" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D62" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E62" s="11" t="inlineStr">
+        <is>
+          <t>DEAD</t>
+        </is>
+      </c>
+      <c r="F62" s="7" t="inlineStr">
+        <is>
+          <t>Shut down June 2024. Listed only so it never reappears in a future version of this file.</t>
+        </is>
+      </c>
+      <c r="G62" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H62" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I62" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="46" customHeight="1">
+      <c r="A63" s="6" t="n">
+        <v>53</v>
+      </c>
+      <c r="B63" s="7" t="inlineStr">
+        <is>
+          <t>Skyray Ventures</t>
+        </is>
+      </c>
+      <c r="C63" s="7" t="inlineStr">
+        <is>
+          <t>Lahore, PK</t>
+        </is>
+      </c>
+      <c r="D63" s="7" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="E63" s="11" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+      <c r="F63" s="7" t="inlineStr">
+        <is>
+          <t>Reviews titled 'Fake Promises'; consistent reports of low pay and micromanagement.</t>
+        </is>
+      </c>
+      <c r="G63" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H63" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I63" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="46" customHeight="1">
+      <c r="A64" s="6" t="n">
+        <v>54</v>
+      </c>
+      <c r="B64" s="7" t="inlineStr">
+        <is>
           <t>Azara Branding</t>
         </is>
       </c>
-      <c r="C51" s="7" t="inlineStr">
+      <c r="C64" s="7" t="inlineStr">
         <is>
           <t>Long Beach, CA</t>
         </is>
       </c>
-      <c r="D51" s="7" t="inlineStr">
+      <c r="D64" s="7" t="inlineStr">
         <is>
           <t>On-site</t>
         </is>
       </c>
-      <c r="E51" s="11" t="inlineStr">
+      <c r="E64" s="11" t="inlineStr">
         <is>
           <t>AVOID</t>
         </is>
       </c>
-      <c r="F51" s="7" t="inlineStr">
-        <is>
-          <t>In-person field and event sales recruiting. Will not build the technical-sales resume you are after.</t>
-        </is>
-      </c>
-      <c r="G51" s="7" t="inlineStr">
+      <c r="F64" s="7" t="inlineStr">
+        <is>
+          <t>Recruits for in-person field and event sales. Will not build the technical-sales resume you are after.</t>
+        </is>
+      </c>
+      <c r="G64" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H51" s="7" t="inlineStr">
+      <c r="H64" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-    </row>
-    <row r="53">
-      <c r="B53" s="15" t="inlineStr">
-        <is>
-          <t>Status key: VERIFIED HIRING = open roles confirmed on the company's own board or a source quoting it, Aug 1 2026 · VERIFIED ACTIVE = company confirmed operating and growing, specific reqs not individually confirmed · ACTIVE = company confirmed real and operating, hiring not individually confirmed · AVOID / DEAD = see the reason in the column to the right.</t>
-        </is>
-      </c>
-    </row>
-    <row r="54"/>
+      <c r="I64" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="B66" s="15" t="inlineStr">
+        <is>
+          <t>Status key: VERIFIED HIRING = open roles confirmed on the company's own board or a source quoting it, Aug 1 2026 · VERIFIED ACTIVE = company confirmed operating and growing, individual reqs not confirmed · ACTIVE = company confirmed real and operating · AIM LATER = real fit, but you are not yet qualified — track it · CUT / DEMOTED = was in v1, removed with the reason stated · AVOID / DEAD = do not spend time. Careers URLs are company-root paths; if one has moved, search the company name plus 'careers' rather than trusting the link.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67"/>
+    <row r="68"/>
   </sheetData>
-  <autoFilter ref="A2:H51"/>
-  <mergeCells count="8">
-    <mergeCell ref="A12:H12"/>
-    <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A19:H19"/>
-    <mergeCell ref="B53:H54"/>
-    <mergeCell ref="A47:H47"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A32:H32"/>
-    <mergeCell ref="A40:H40"/>
+  <autoFilter ref="A2:I64"/>
+  <mergeCells count="10">
+    <mergeCell ref="A43:I43"/>
+    <mergeCell ref="B66:I68"/>
+    <mergeCell ref="A60:I60"/>
+    <mergeCell ref="A32:I32"/>
+    <mergeCell ref="A13:I13"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A3:I3"/>
+    <mergeCell ref="A53:I53"/>
+    <mergeCell ref="A26:I26"/>
+    <mergeCell ref="A21:I21"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H27" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H29" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H30" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H31" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H33" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H34" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H35" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H36" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H37" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H38" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H39" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H41" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H42" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H43" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H44" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H45" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H46" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I4" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I12" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I16" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I28" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I29" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I30" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I31" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I33" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I34" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I35" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I36" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I37" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I38" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I39" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I40" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I41" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I42" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I44" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I45" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I46" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I47" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I48" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I49" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I50" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I51" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I52" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I58" r:id="rId45"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>